<commit_message>
Add issuer info fields, tax-exclusive line items with consumption tax calc, and floor rounding
Rebuilt template.xlsx layout to match user-provided real estimate template
(title/client/issuer blocks, item table at row 17-29, subtotal/tax/total rows)
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -16,8 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy年mm月dd日"/>
+    <numFmt numFmtId="165" formatCode="#,##0&quot;円（税込）&quot;"/>
+  </numFmts>
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,7 +33,21 @@
       <sz val="20"/>
     </font>
     <font>
+      <sz val="14"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
+    <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="3">
@@ -72,14 +89,54 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,159 +502,161 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>御 見 積 書</t>
-        </is>
-      </c>
-    </row>
+          <t>御　見　積　書</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>○○○○ 様</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>発行日：</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>（宛先を入力）</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>様</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>件名：</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>見積番号：</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>品名</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>規格・仕様</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>単位</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>数量</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>単価</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>金額</t>
-        </is>
-      </c>
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="K4" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="I6" s="6" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>下記の通りお見積申し上げますので何卒宜しくお願い致します。</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
+      <c r="K9" s="8" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
+      <c r="N10" s="8" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
+      <c r="N11" s="8" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n"/>
+      <c r="N12" s="8" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n"/>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>見積金額</t>
+        </is>
+      </c>
       <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
+      <c r="E13" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
+      <c r="L13" s="9" t="inlineStr">
+        <is>
+          <t>検　印</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="n"/>
+      <c r="N13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n"/>
-      <c r="B14" s="3" t="n"/>
       <c r="C14" s="3" t="n"/>
       <c r="D14" s="3" t="n"/>
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="n"/>
+      <c r="G14" s="3" t="n"/>
+      <c r="L14" s="3" t="inlineStr"/>
+      <c r="M14" s="3" t="inlineStr"/>
+      <c r="N14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n"/>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
+      <c r="L15" s="3" t="n"/>
+      <c r="M15" s="3" t="n"/>
+      <c r="N15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n"/>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
+      <c r="L16" s="3" t="n"/>
+      <c r="M16" s="3" t="n"/>
+      <c r="N16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n"/>
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>寸法・規格</t>
+        </is>
+      </c>
       <c r="E17" s="3" t="n"/>
       <c r="F17" s="3" t="n"/>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="H17" s="11" t="inlineStr">
+        <is>
+          <t>単位</t>
+        </is>
+      </c>
+      <c r="I17" s="11" t="inlineStr">
+        <is>
+          <t>単価</t>
+        </is>
+      </c>
+      <c r="J17" s="11" t="inlineStr">
+        <is>
+          <t>金額</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="11" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="n"/>
+      <c r="N17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -606,6 +665,14 @@
       <c r="D18" s="3" t="n"/>
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="3" t="n"/>
+      <c r="G18" s="3" t="n"/>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="3" t="n"/>
+      <c r="J18" s="3" t="n"/>
+      <c r="K18" s="3" t="n"/>
+      <c r="L18" s="3" t="n"/>
+      <c r="M18" s="3" t="n"/>
+      <c r="N18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
@@ -614,6 +681,14 @@
       <c r="D19" s="3" t="n"/>
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="3" t="n"/>
+      <c r="G19" s="3" t="n"/>
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="n"/>
+      <c r="J19" s="3" t="n"/>
+      <c r="K19" s="3" t="n"/>
+      <c r="L19" s="3" t="n"/>
+      <c r="M19" s="3" t="n"/>
+      <c r="N19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -622,6 +697,14 @@
       <c r="D20" s="3" t="n"/>
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
+      <c r="G20" s="3" t="n"/>
+      <c r="H20" s="3" t="n"/>
+      <c r="I20" s="3" t="n"/>
+      <c r="J20" s="3" t="n"/>
+      <c r="K20" s="3" t="n"/>
+      <c r="L20" s="3" t="n"/>
+      <c r="M20" s="3" t="n"/>
+      <c r="N20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -630,6 +713,14 @@
       <c r="D21" s="3" t="n"/>
       <c r="E21" s="3" t="n"/>
       <c r="F21" s="3" t="n"/>
+      <c r="G21" s="3" t="n"/>
+      <c r="H21" s="3" t="n"/>
+      <c r="I21" s="3" t="n"/>
+      <c r="J21" s="3" t="n"/>
+      <c r="K21" s="3" t="n"/>
+      <c r="L21" s="3" t="n"/>
+      <c r="M21" s="3" t="n"/>
+      <c r="N21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -638,6 +729,14 @@
       <c r="D22" s="3" t="n"/>
       <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="n"/>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="n"/>
+      <c r="K22" s="3" t="n"/>
+      <c r="L22" s="3" t="n"/>
+      <c r="M22" s="3" t="n"/>
+      <c r="N22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -646,6 +745,14 @@
       <c r="D23" s="3" t="n"/>
       <c r="E23" s="3" t="n"/>
       <c r="F23" s="3" t="n"/>
+      <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="n"/>
+      <c r="I23" s="3" t="n"/>
+      <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
+      <c r="L23" s="3" t="n"/>
+      <c r="M23" s="3" t="n"/>
+      <c r="N23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -654,6 +761,14 @@
       <c r="D24" s="3" t="n"/>
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
+      <c r="G24" s="3" t="n"/>
+      <c r="H24" s="3" t="n"/>
+      <c r="I24" s="3" t="n"/>
+      <c r="J24" s="3" t="n"/>
+      <c r="K24" s="3" t="n"/>
+      <c r="L24" s="3" t="n"/>
+      <c r="M24" s="3" t="n"/>
+      <c r="N24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
@@ -662,6 +777,14 @@
       <c r="D25" s="3" t="n"/>
       <c r="E25" s="3" t="n"/>
       <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
+      <c r="I25" s="3" t="n"/>
+      <c r="J25" s="3" t="n"/>
+      <c r="K25" s="3" t="n"/>
+      <c r="L25" s="3" t="n"/>
+      <c r="M25" s="3" t="n"/>
+      <c r="N25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -670,6 +793,14 @@
       <c r="D26" s="3" t="n"/>
       <c r="E26" s="3" t="n"/>
       <c r="F26" s="3" t="n"/>
+      <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="n"/>
+      <c r="J26" s="3" t="n"/>
+      <c r="K26" s="3" t="n"/>
+      <c r="L26" s="3" t="n"/>
+      <c r="M26" s="3" t="n"/>
+      <c r="N26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
@@ -678,15 +809,193 @@
       <c r="D27" s="3" t="n"/>
       <c r="E27" s="3" t="n"/>
       <c r="F27" s="3" t="n"/>
+      <c r="G27" s="3" t="n"/>
+      <c r="H27" s="3" t="n"/>
+      <c r="I27" s="3" t="n"/>
+      <c r="J27" s="3" t="n"/>
+      <c r="K27" s="3" t="n"/>
+      <c r="L27" s="3" t="n"/>
+      <c r="M27" s="3" t="n"/>
+      <c r="N27" s="3" t="n"/>
     </row>
     <row r="28">
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>合計</t>
-        </is>
-      </c>
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="3" t="n"/>
+      <c r="C28" s="3" t="n"/>
+      <c r="D28" s="3" t="n"/>
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="3" t="n"/>
+      <c r="G28" s="3" t="n"/>
+      <c r="H28" s="3" t="n"/>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+      <c r="K28" s="3" t="n"/>
+      <c r="L28" s="3" t="n"/>
+      <c r="M28" s="3" t="n"/>
+      <c r="N28" s="3" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="3" t="n"/>
+      <c r="C29" s="3" t="n"/>
+      <c r="D29" s="3" t="n"/>
+      <c r="E29" s="3" t="n"/>
+      <c r="F29" s="3" t="n"/>
+      <c r="G29" s="3" t="n"/>
+      <c r="H29" s="3" t="n"/>
+      <c r="I29" s="3" t="n"/>
+      <c r="J29" s="3" t="n"/>
+      <c r="K29" s="3" t="n"/>
+      <c r="L29" s="3" t="n"/>
+      <c r="M29" s="3" t="n"/>
+      <c r="N29" s="3" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>小　計</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n"/>
+      <c r="C31" s="3" t="n"/>
+      <c r="D31" s="3" t="n"/>
+      <c r="E31" s="3" t="n"/>
+      <c r="F31" s="3" t="n"/>
+      <c r="J31" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="3" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>消　費　税</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n"/>
+      <c r="C32" s="3" t="n"/>
+      <c r="D32" s="3" t="n"/>
+      <c r="E32" s="3" t="n"/>
+      <c r="F32" s="3" t="n"/>
+      <c r="G32" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="H32" s="14" t="inlineStr">
+        <is>
+          <t>％</t>
+        </is>
+      </c>
+      <c r="J32" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="3" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>合　計</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n"/>
+      <c r="C33" s="3" t="n"/>
+      <c r="D33" s="3" t="n"/>
+      <c r="E33" s="3" t="n"/>
+      <c r="F33" s="3" t="n"/>
+      <c r="G33" s="3" t="n"/>
+      <c r="H33" s="3" t="n"/>
+      <c r="I33" s="3" t="n"/>
+      <c r="J33" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="3" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n"/>
+      <c r="B34" s="3" t="n"/>
+      <c r="C34" s="3" t="n"/>
+      <c r="D34" s="3" t="n"/>
+      <c r="E34" s="3" t="n"/>
+      <c r="F34" s="3" t="n"/>
+      <c r="G34" s="3" t="n"/>
+      <c r="H34" s="3" t="n"/>
+      <c r="I34" s="3" t="n"/>
+      <c r="J34" s="3" t="n"/>
+      <c r="K34" s="3" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="71">
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="L24:N24"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="L18:N18"/>
+    <mergeCell ref="L23:N23"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="M14:M16"/>
+    <mergeCell ref="L20:N20"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="L26:N26"/>
+    <mergeCell ref="L29:N29"/>
+    <mergeCell ref="K4:N4"/>
+    <mergeCell ref="L25:N25"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="L22:N22"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A3:D4"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="E13:G14"/>
+    <mergeCell ref="C13:D14"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="K9:N9"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="L21:N21"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="J33:K34"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="L27:N27"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="L17:N17"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="I6:N6"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A1:N2"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="L28:N28"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="L13:N13"/>
+    <mergeCell ref="L19:N19"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="K8:N8"/>
+    <mergeCell ref="L14:L16"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="A33:I34"/>
+    <mergeCell ref="N14:N16"/>
+    <mergeCell ref="J17:K17"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix unstyled gap row when items overflow, and add missing unit (単位) field
- The row between the pre-formatted data block and the old subtotal
  position was never styled during overflow handling, leaving it
  without borders/merges/fonts (visible as broken formatting).
  Styling now covers the full contiguous range with no gap.
- 単位 was parsed nowhere and never written to the template; now
  extracted from PDF tables, Excel, editable in the UI, and filled
  into the template's unit column.
- Added thousand-separator number format to price/amount data cells.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -20,7 +20,7 @@
     <numFmt numFmtId="164" formatCode="yyyy年mm月dd日"/>
     <numFmt numFmtId="165" formatCode="#,##0&quot;円（税込）&quot;"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,6 +44,9 @@
     <font>
       <b val="1"/>
       <sz val="16"/>
+    </font>
+    <font>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -89,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -122,6 +125,12 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -131,10 +140,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -659,199 +668,199 @@
       <c r="N17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n"/>
+      <c r="A18" s="12" t="n"/>
       <c r="B18" s="3" t="n"/>
       <c r="C18" s="3" t="n"/>
-      <c r="D18" s="3" t="n"/>
+      <c r="D18" s="12" t="n"/>
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="3" t="n"/>
-      <c r="G18" s="3" t="n"/>
-      <c r="H18" s="3" t="n"/>
-      <c r="I18" s="3" t="n"/>
-      <c r="J18" s="3" t="n"/>
+      <c r="G18" s="12" t="n"/>
+      <c r="H18" s="12" t="n"/>
+      <c r="I18" s="13" t="n"/>
+      <c r="J18" s="13" t="n"/>
       <c r="K18" s="3" t="n"/>
-      <c r="L18" s="3" t="n"/>
+      <c r="L18" s="12" t="n"/>
       <c r="M18" s="3" t="n"/>
       <c r="N18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n"/>
+      <c r="A19" s="12" t="n"/>
       <c r="B19" s="3" t="n"/>
       <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
+      <c r="D19" s="12" t="n"/>
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="n"/>
-      <c r="J19" s="3" t="n"/>
+      <c r="G19" s="12" t="n"/>
+      <c r="H19" s="12" t="n"/>
+      <c r="I19" s="13" t="n"/>
+      <c r="J19" s="13" t="n"/>
       <c r="K19" s="3" t="n"/>
-      <c r="L19" s="3" t="n"/>
+      <c r="L19" s="12" t="n"/>
       <c r="M19" s="3" t="n"/>
       <c r="N19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n"/>
+      <c r="A20" s="12" t="n"/>
       <c r="B20" s="3" t="n"/>
       <c r="C20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
+      <c r="D20" s="12" t="n"/>
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="n"/>
-      <c r="J20" s="3" t="n"/>
+      <c r="G20" s="12" t="n"/>
+      <c r="H20" s="12" t="n"/>
+      <c r="I20" s="13" t="n"/>
+      <c r="J20" s="13" t="n"/>
       <c r="K20" s="3" t="n"/>
-      <c r="L20" s="3" t="n"/>
+      <c r="L20" s="12" t="n"/>
       <c r="M20" s="3" t="n"/>
       <c r="N20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n"/>
+      <c r="A21" s="12" t="n"/>
       <c r="B21" s="3" t="n"/>
       <c r="C21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
+      <c r="D21" s="12" t="n"/>
       <c r="E21" s="3" t="n"/>
       <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3" t="n"/>
-      <c r="J21" s="3" t="n"/>
+      <c r="G21" s="12" t="n"/>
+      <c r="H21" s="12" t="n"/>
+      <c r="I21" s="13" t="n"/>
+      <c r="J21" s="13" t="n"/>
       <c r="K21" s="3" t="n"/>
-      <c r="L21" s="3" t="n"/>
+      <c r="L21" s="12" t="n"/>
       <c r="M21" s="3" t="n"/>
       <c r="N21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n"/>
+      <c r="A22" s="12" t="n"/>
       <c r="B22" s="3" t="n"/>
       <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
+      <c r="D22" s="12" t="n"/>
       <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="n"/>
+      <c r="G22" s="12" t="n"/>
+      <c r="H22" s="12" t="n"/>
+      <c r="I22" s="13" t="n"/>
+      <c r="J22" s="13" t="n"/>
       <c r="K22" s="3" t="n"/>
-      <c r="L22" s="3" t="n"/>
+      <c r="L22" s="12" t="n"/>
       <c r="M22" s="3" t="n"/>
       <c r="N22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n"/>
+      <c r="A23" s="12" t="n"/>
       <c r="B23" s="3" t="n"/>
       <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
+      <c r="D23" s="12" t="n"/>
       <c r="E23" s="3" t="n"/>
       <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="3" t="n"/>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="12" t="n"/>
+      <c r="I23" s="13" t="n"/>
+      <c r="J23" s="13" t="n"/>
       <c r="K23" s="3" t="n"/>
-      <c r="L23" s="3" t="n"/>
+      <c r="L23" s="12" t="n"/>
       <c r="M23" s="3" t="n"/>
       <c r="N23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n"/>
+      <c r="A24" s="12" t="n"/>
       <c r="B24" s="3" t="n"/>
       <c r="C24" s="3" t="n"/>
-      <c r="D24" s="3" t="n"/>
+      <c r="D24" s="12" t="n"/>
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="3" t="n"/>
-      <c r="J24" s="3" t="n"/>
+      <c r="G24" s="12" t="n"/>
+      <c r="H24" s="12" t="n"/>
+      <c r="I24" s="13" t="n"/>
+      <c r="J24" s="13" t="n"/>
       <c r="K24" s="3" t="n"/>
-      <c r="L24" s="3" t="n"/>
+      <c r="L24" s="12" t="n"/>
       <c r="M24" s="3" t="n"/>
       <c r="N24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n"/>
+      <c r="A25" s="12" t="n"/>
       <c r="B25" s="3" t="n"/>
       <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
+      <c r="D25" s="12" t="n"/>
       <c r="E25" s="3" t="n"/>
       <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n"/>
-      <c r="I25" s="3" t="n"/>
-      <c r="J25" s="3" t="n"/>
+      <c r="G25" s="12" t="n"/>
+      <c r="H25" s="12" t="n"/>
+      <c r="I25" s="13" t="n"/>
+      <c r="J25" s="13" t="n"/>
       <c r="K25" s="3" t="n"/>
-      <c r="L25" s="3" t="n"/>
+      <c r="L25" s="12" t="n"/>
       <c r="M25" s="3" t="n"/>
       <c r="N25" s="3" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n"/>
+      <c r="A26" s="12" t="n"/>
       <c r="B26" s="3" t="n"/>
       <c r="C26" s="3" t="n"/>
-      <c r="D26" s="3" t="n"/>
+      <c r="D26" s="12" t="n"/>
       <c r="E26" s="3" t="n"/>
       <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="n"/>
-      <c r="I26" s="3" t="n"/>
-      <c r="J26" s="3" t="n"/>
+      <c r="G26" s="12" t="n"/>
+      <c r="H26" s="12" t="n"/>
+      <c r="I26" s="13" t="n"/>
+      <c r="J26" s="13" t="n"/>
       <c r="K26" s="3" t="n"/>
-      <c r="L26" s="3" t="n"/>
+      <c r="L26" s="12" t="n"/>
       <c r="M26" s="3" t="n"/>
       <c r="N26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n"/>
+      <c r="A27" s="12" t="n"/>
       <c r="B27" s="3" t="n"/>
       <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
+      <c r="D27" s="12" t="n"/>
       <c r="E27" s="3" t="n"/>
       <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="n"/>
-      <c r="I27" s="3" t="n"/>
-      <c r="J27" s="3" t="n"/>
+      <c r="G27" s="12" t="n"/>
+      <c r="H27" s="12" t="n"/>
+      <c r="I27" s="13" t="n"/>
+      <c r="J27" s="13" t="n"/>
       <c r="K27" s="3" t="n"/>
-      <c r="L27" s="3" t="n"/>
+      <c r="L27" s="12" t="n"/>
       <c r="M27" s="3" t="n"/>
       <c r="N27" s="3" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="n"/>
+      <c r="A28" s="12" t="n"/>
       <c r="B28" s="3" t="n"/>
       <c r="C28" s="3" t="n"/>
-      <c r="D28" s="3" t="n"/>
+      <c r="D28" s="12" t="n"/>
       <c r="E28" s="3" t="n"/>
       <c r="F28" s="3" t="n"/>
-      <c r="G28" s="3" t="n"/>
-      <c r="H28" s="3" t="n"/>
-      <c r="I28" s="3" t="n"/>
-      <c r="J28" s="3" t="n"/>
+      <c r="G28" s="12" t="n"/>
+      <c r="H28" s="12" t="n"/>
+      <c r="I28" s="13" t="n"/>
+      <c r="J28" s="13" t="n"/>
       <c r="K28" s="3" t="n"/>
-      <c r="L28" s="3" t="n"/>
+      <c r="L28" s="12" t="n"/>
       <c r="M28" s="3" t="n"/>
       <c r="N28" s="3" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n"/>
+      <c r="A29" s="12" t="n"/>
       <c r="B29" s="3" t="n"/>
       <c r="C29" s="3" t="n"/>
-      <c r="D29" s="3" t="n"/>
+      <c r="D29" s="12" t="n"/>
       <c r="E29" s="3" t="n"/>
       <c r="F29" s="3" t="n"/>
-      <c r="G29" s="3" t="n"/>
-      <c r="H29" s="3" t="n"/>
-      <c r="I29" s="3" t="n"/>
-      <c r="J29" s="3" t="n"/>
+      <c r="G29" s="12" t="n"/>
+      <c r="H29" s="12" t="n"/>
+      <c r="I29" s="13" t="n"/>
+      <c r="J29" s="13" t="n"/>
       <c r="K29" s="3" t="n"/>
-      <c r="L29" s="3" t="n"/>
+      <c r="L29" s="12" t="n"/>
       <c r="M29" s="3" t="n"/>
       <c r="N29" s="3" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="A31" s="14" t="inlineStr">
         <is>
           <t>小　計</t>
         </is>
@@ -861,13 +870,13 @@
       <c r="D31" s="3" t="n"/>
       <c r="E31" s="3" t="n"/>
       <c r="F31" s="3" t="n"/>
-      <c r="J31" s="13" t="n">
+      <c r="J31" s="15" t="n">
         <v>0</v>
       </c>
       <c r="K31" s="3" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="inlineStr">
+      <c r="A32" s="14" t="inlineStr">
         <is>
           <t>消　費　税</t>
         </is>
@@ -877,21 +886,21 @@
       <c r="D32" s="3" t="n"/>
       <c r="E32" s="3" t="n"/>
       <c r="F32" s="3" t="n"/>
-      <c r="G32" s="14" t="n">
+      <c r="G32" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="H32" s="14" t="inlineStr">
+      <c r="H32" s="16" t="inlineStr">
         <is>
           <t>％</t>
         </is>
       </c>
-      <c r="J32" s="13" t="n">
+      <c r="J32" s="15" t="n">
         <v>0</v>
       </c>
       <c r="K32" s="3" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>合　計</t>
         </is>
@@ -904,7 +913,7 @@
       <c r="G33" s="3" t="n"/>
       <c r="H33" s="3" t="n"/>
       <c r="I33" s="3" t="n"/>
-      <c r="J33" s="16" t="n">
+      <c r="J33" s="18" t="n">
         <v>0</v>
       </c>
       <c r="K33" s="3" t="n"/>

</xml_diff>

<commit_message>
Add invoice (請求書) output alongside the quote (見積書)
- template.xlsx now has two sheets built from a shared layout
  function: 見積書 and 請求書 (title/greeting/amount-label differ;
  請求書 also gets a 振込先 (bank transfer) row, matching the
  reference 請求書 sheet from the user's sample workbook).
- fill_template gains document_type and bank_info params; overflow
  handling now also accounts for and relocates the bank row.
- Issuer profiles (saved/recalled by company name) now include
  bank_info, editable and reused for the invoice download.
- Two separate download buttons: 見積書 and 請求書, both generated
  from the same item list/markup/tax inputs.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="見積書" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="請求書" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -92,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -145,6 +146,12 @@
     </xf>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1007,4 +1014,517 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>御　請　求　書</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>（宛先を入力）</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>様</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="K4" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="I6" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>下記の通りご請求申し上げますので何卒宜しくお願い致します。</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="K9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="N10" s="8" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="N11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="N12" s="8" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>請求金額</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
+      <c r="L13" s="9" t="inlineStr">
+        <is>
+          <t>検　印</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="n"/>
+      <c r="N13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="n"/>
+      <c r="G14" s="3" t="n"/>
+      <c r="L14" s="3" t="inlineStr"/>
+      <c r="M14" s="3" t="inlineStr"/>
+      <c r="N14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="L15" s="3" t="n"/>
+      <c r="M15" s="3" t="n"/>
+      <c r="N15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="L16" s="3" t="n"/>
+      <c r="M16" s="3" t="n"/>
+      <c r="N16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>寸法・規格</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="H17" s="11" t="inlineStr">
+        <is>
+          <t>単位</t>
+        </is>
+      </c>
+      <c r="I17" s="11" t="inlineStr">
+        <is>
+          <t>単価</t>
+        </is>
+      </c>
+      <c r="J17" s="11" t="inlineStr">
+        <is>
+          <t>金額</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="11" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="n"/>
+      <c r="N17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="n"/>
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="12" t="n"/>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="3" t="n"/>
+      <c r="G18" s="12" t="n"/>
+      <c r="H18" s="12" t="n"/>
+      <c r="I18" s="13" t="n"/>
+      <c r="J18" s="13" t="n"/>
+      <c r="K18" s="3" t="n"/>
+      <c r="L18" s="12" t="n"/>
+      <c r="M18" s="3" t="n"/>
+      <c r="N18" s="3" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n"/>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="3" t="n"/>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
+      <c r="G19" s="12" t="n"/>
+      <c r="H19" s="12" t="n"/>
+      <c r="I19" s="13" t="n"/>
+      <c r="J19" s="13" t="n"/>
+      <c r="K19" s="3" t="n"/>
+      <c r="L19" s="12" t="n"/>
+      <c r="M19" s="3" t="n"/>
+      <c r="N19" s="3" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="n"/>
+      <c r="B20" s="3" t="n"/>
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="3" t="n"/>
+      <c r="F20" s="3" t="n"/>
+      <c r="G20" s="12" t="n"/>
+      <c r="H20" s="12" t="n"/>
+      <c r="I20" s="13" t="n"/>
+      <c r="J20" s="13" t="n"/>
+      <c r="K20" s="3" t="n"/>
+      <c r="L20" s="12" t="n"/>
+      <c r="M20" s="3" t="n"/>
+      <c r="N20" s="3" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n"/>
+      <c r="B21" s="3" t="n"/>
+      <c r="C21" s="3" t="n"/>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="3" t="n"/>
+      <c r="G21" s="12" t="n"/>
+      <c r="H21" s="12" t="n"/>
+      <c r="I21" s="13" t="n"/>
+      <c r="J21" s="13" t="n"/>
+      <c r="K21" s="3" t="n"/>
+      <c r="L21" s="12" t="n"/>
+      <c r="M21" s="3" t="n"/>
+      <c r="N21" s="3" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="n"/>
+      <c r="B22" s="3" t="n"/>
+      <c r="C22" s="3" t="n"/>
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
+      <c r="G22" s="12" t="n"/>
+      <c r="H22" s="12" t="n"/>
+      <c r="I22" s="13" t="n"/>
+      <c r="J22" s="13" t="n"/>
+      <c r="K22" s="3" t="n"/>
+      <c r="L22" s="12" t="n"/>
+      <c r="M22" s="3" t="n"/>
+      <c r="N22" s="3" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n"/>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="12" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="12" t="n"/>
+      <c r="I23" s="13" t="n"/>
+      <c r="J23" s="13" t="n"/>
+      <c r="K23" s="3" t="n"/>
+      <c r="L23" s="12" t="n"/>
+      <c r="M23" s="3" t="n"/>
+      <c r="N23" s="3" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n"/>
+      <c r="B24" s="3" t="n"/>
+      <c r="C24" s="3" t="n"/>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="3" t="n"/>
+      <c r="F24" s="3" t="n"/>
+      <c r="G24" s="12" t="n"/>
+      <c r="H24" s="12" t="n"/>
+      <c r="I24" s="13" t="n"/>
+      <c r="J24" s="13" t="n"/>
+      <c r="K24" s="3" t="n"/>
+      <c r="L24" s="12" t="n"/>
+      <c r="M24" s="3" t="n"/>
+      <c r="N24" s="3" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n"/>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="12" t="n"/>
+      <c r="H25" s="12" t="n"/>
+      <c r="I25" s="13" t="n"/>
+      <c r="J25" s="13" t="n"/>
+      <c r="K25" s="3" t="n"/>
+      <c r="L25" s="12" t="n"/>
+      <c r="M25" s="3" t="n"/>
+      <c r="N25" s="3" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n"/>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="12" t="n"/>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
+      <c r="G26" s="12" t="n"/>
+      <c r="H26" s="12" t="n"/>
+      <c r="I26" s="13" t="n"/>
+      <c r="J26" s="13" t="n"/>
+      <c r="K26" s="3" t="n"/>
+      <c r="L26" s="12" t="n"/>
+      <c r="M26" s="3" t="n"/>
+      <c r="N26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n"/>
+      <c r="B27" s="3" t="n"/>
+      <c r="C27" s="3" t="n"/>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="3" t="n"/>
+      <c r="F27" s="3" t="n"/>
+      <c r="G27" s="12" t="n"/>
+      <c r="H27" s="12" t="n"/>
+      <c r="I27" s="13" t="n"/>
+      <c r="J27" s="13" t="n"/>
+      <c r="K27" s="3" t="n"/>
+      <c r="L27" s="12" t="n"/>
+      <c r="M27" s="3" t="n"/>
+      <c r="N27" s="3" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="n"/>
+      <c r="B28" s="3" t="n"/>
+      <c r="C28" s="3" t="n"/>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="3" t="n"/>
+      <c r="G28" s="12" t="n"/>
+      <c r="H28" s="12" t="n"/>
+      <c r="I28" s="13" t="n"/>
+      <c r="J28" s="13" t="n"/>
+      <c r="K28" s="3" t="n"/>
+      <c r="L28" s="12" t="n"/>
+      <c r="M28" s="3" t="n"/>
+      <c r="N28" s="3" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n"/>
+      <c r="B29" s="3" t="n"/>
+      <c r="C29" s="3" t="n"/>
+      <c r="D29" s="12" t="n"/>
+      <c r="E29" s="3" t="n"/>
+      <c r="F29" s="3" t="n"/>
+      <c r="G29" s="12" t="n"/>
+      <c r="H29" s="12" t="n"/>
+      <c r="I29" s="13" t="n"/>
+      <c r="J29" s="13" t="n"/>
+      <c r="K29" s="3" t="n"/>
+      <c r="L29" s="12" t="n"/>
+      <c r="M29" s="3" t="n"/>
+      <c r="N29" s="3" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>小　計</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n"/>
+      <c r="C31" s="3" t="n"/>
+      <c r="D31" s="3" t="n"/>
+      <c r="E31" s="3" t="n"/>
+      <c r="F31" s="3" t="n"/>
+      <c r="J31" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="3" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>消　費　税</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n"/>
+      <c r="C32" s="3" t="n"/>
+      <c r="D32" s="3" t="n"/>
+      <c r="E32" s="3" t="n"/>
+      <c r="F32" s="3" t="n"/>
+      <c r="G32" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="H32" s="16" t="inlineStr">
+        <is>
+          <t>％</t>
+        </is>
+      </c>
+      <c r="J32" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="3" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>合　計</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n"/>
+      <c r="C33" s="3" t="n"/>
+      <c r="D33" s="3" t="n"/>
+      <c r="E33" s="3" t="n"/>
+      <c r="F33" s="3" t="n"/>
+      <c r="G33" s="3" t="n"/>
+      <c r="H33" s="3" t="n"/>
+      <c r="I33" s="3" t="n"/>
+      <c r="J33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="3" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n"/>
+      <c r="B34" s="3" t="n"/>
+      <c r="C34" s="3" t="n"/>
+      <c r="D34" s="3" t="n"/>
+      <c r="E34" s="3" t="n"/>
+      <c r="F34" s="3" t="n"/>
+      <c r="G34" s="3" t="n"/>
+      <c r="H34" s="3" t="n"/>
+      <c r="I34" s="3" t="n"/>
+      <c r="J34" s="3" t="n"/>
+      <c r="K34" s="3" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>振込先</t>
+        </is>
+      </c>
+      <c r="C35" s="20" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="72">
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="L24:N24"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="L18:N18"/>
+    <mergeCell ref="L23:N23"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="M14:M16"/>
+    <mergeCell ref="L20:N20"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="L26:N26"/>
+    <mergeCell ref="L29:N29"/>
+    <mergeCell ref="K4:N4"/>
+    <mergeCell ref="L25:N25"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="L22:N22"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A3:D4"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="E13:G14"/>
+    <mergeCell ref="C13:D14"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="K9:N9"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="L21:N21"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="J33:K34"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="L27:N27"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="L17:N17"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="I6:N6"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A1:N2"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="L28:N28"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="L13:N13"/>
+    <mergeCell ref="L19:N19"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="K8:N8"/>
+    <mergeCell ref="L14:L16"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="A33:I34"/>
+    <mergeCell ref="N14:N16"/>
+    <mergeCell ref="C35:N35"/>
+    <mergeCell ref="J17:K17"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>